<commit_message>
Bieu mau thu thap du lieu: bo o Chu tich Cong doan (cong doan co so truong cong lap ket thuc 01/6/2025); AT06 bo phan cap = Van phong
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bieu-mau/thu-thap-du-lieu-truong.xlsx
+++ b/bieu-mau/thu-thap-du-lieu-truong.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'0. HƯỚNG DẪN'!$A$1:$E$29</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'1. Thông tin trường'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'1. Thông tin trường'!$A$1:$D$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'1. Thông tin trường'!$A$1:$D$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'2. Điểm trường &amp; Lớp học'!$15:$15</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'2. Điểm trường &amp; Lớp học'!$A$1:$L$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'3. Email đăng nhập'!$4:$4</definedName>
@@ -889,6 +889,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1378,7 +1379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1401,6 +1402,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="28" t="inlineStr">
         <is>
@@ -1774,12 +1776,12 @@
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="31" t="inlineStr">
         <is>
-          <t>CT_CONG_DOAN</t>
+          <t>TPT_DOI</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Chủ tịch Công đoàn</t>
+          <t>Tổng phụ trách Đội</t>
         </is>
       </c>
       <c r="C27" s="32" t="inlineStr"/>
@@ -1788,210 +1790,210 @@
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="31" t="inlineStr">
         <is>
-          <t>TPT_DOI</t>
+          <t>TRUONG_BAN_CMHS</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Tổng phụ trách Đội</t>
+          <t>Trưởng ban đại diện cha mẹ học sinh</t>
         </is>
       </c>
       <c r="C28" s="32" t="inlineStr"/>
       <c r="D28" s="11" t="inlineStr"/>
     </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="31" t="inlineStr">
-        <is>
-          <t>TRUONG_BAN_CMHS</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Trưởng ban đại diện cha mẹ học sinh</t>
-        </is>
-      </c>
-      <c r="C29" s="32" t="inlineStr"/>
-      <c r="D29" s="11" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>C. TÌNH TRẠNG TRƯỜNG CHUẨN QUỐC GIA</t>
         </is>
       </c>
-      <c r="B30" s="16" t="n"/>
-      <c r="C30" s="16" t="n"/>
-      <c r="D30" s="17" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="17" t="n"/>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>CNQG_MUC_DO</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Mức đạt chuẩn quốc gia hiện tại</t>
+        </is>
+      </c>
+      <c r="C30" s="32" t="inlineStr"/>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Chọn trong danh sách</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="31" t="inlineStr">
         <is>
-          <t>CNQG_MUC_DO</t>
+          <t>CNQG_SO_QD</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Mức đạt chuẩn quốc gia hiện tại</t>
+          <t>Số quyết định công nhận</t>
         </is>
       </c>
       <c r="C31" s="32" t="inlineStr"/>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>Chọn trong danh sách</t>
-        </is>
-      </c>
+      <c r="D31" s="11" t="inlineStr"/>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="31" t="inlineStr">
         <is>
-          <t>CNQG_SO_QD</t>
+          <t>CNQG_NGAY_KY</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Số quyết định công nhận</t>
+          <t>Ngày ký quyết định công nhận</t>
         </is>
       </c>
       <c r="C32" s="32" t="inlineStr"/>
-      <c r="D32" s="11" t="inlineStr"/>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>dd/mm/yyyy</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
-          <t>CNQG_NGAY_KY</t>
+          <t>CNQG_HET_HAN</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Ngày ký quyết định công nhận</t>
+          <t>Ngày hết hạn công nhận</t>
         </is>
       </c>
       <c r="C33" s="32" t="inlineStr"/>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>dd/mm/yyyy</t>
+          <t>Thường 5 năm kể từ ngày ký</t>
         </is>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="31" t="inlineStr">
         <is>
-          <t>CNQG_HET_HAN</t>
+          <t>CO_HOI_DONG_TDG</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Ngày hết hạn công nhận</t>
+          <t>Đã lập Hội đồng tự đánh giá chưa</t>
         </is>
       </c>
       <c r="C34" s="32" t="inlineStr"/>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Thường 5 năm kể từ ngày ký</t>
+          <t>Chọn Có / Không</t>
         </is>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="31" t="inlineStr">
         <is>
-          <t>CO_HOI_DONG_TDG</t>
+          <t>QD_HOI_DONG_TDG</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Đã lập Hội đồng tự đánh giá chưa</t>
+          <t>Số, ngày QĐ thành lập Hội đồng TĐG</t>
         </is>
       </c>
       <c r="C35" s="32" t="inlineStr"/>
-      <c r="D35" s="11" t="inlineStr">
-        <is>
-          <t>Chọn Có / Không</t>
-        </is>
-      </c>
+      <c r="D35" s="11" t="inlineStr"/>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="31" t="inlineStr">
         <is>
-          <t>QD_HOI_DONG_TDG</t>
+          <t>BC_TDG_GAN_NHAT</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Số, ngày QĐ thành lập Hội đồng TĐG</t>
+          <t>Năm học của báo cáo TĐG gần nhất</t>
         </is>
       </c>
       <c r="C36" s="32" t="inlineStr"/>
       <c r="D36" s="11" t="inlineStr"/>
     </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="31" t="inlineStr">
-        <is>
-          <t>BC_TDG_GAN_NHAT</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Năm học của báo cáo TĐG gần nhất</t>
-        </is>
-      </c>
-      <c r="C37" s="32" t="inlineStr"/>
-      <c r="D37" s="11" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>D. QUY MÔ NĂM HỌC HIỆN TẠI</t>
         </is>
       </c>
-      <c r="B38" s="16" t="n"/>
-      <c r="C38" s="16" t="n"/>
-      <c r="D38" s="17" t="n"/>
+      <c r="B37" s="16" t="n"/>
+      <c r="C37" s="16" t="n"/>
+      <c r="D37" s="17" t="n"/>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>NAM_HOC</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Năm học hiện tại</t>
+        </is>
+      </c>
+      <c r="C38" s="32" t="inlineStr"/>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>2026-2027</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="31" t="inlineStr">
         <is>
-          <t>NAM_HOC</t>
+          <t>SO_LOP</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Năm học hiện tại</t>
+          <t>Tổng số lớp</t>
         </is>
       </c>
       <c r="C39" s="32" t="inlineStr"/>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>2026-2027</t>
+          <t>Để đối chiếu với tệp CSDL ngành</t>
         </is>
       </c>
     </row>
     <row r="40" ht="24" customHeight="1">
       <c r="A40" s="31" t="inlineStr">
         <is>
-          <t>SO_LOP</t>
+          <t>SO_HOC_SINH</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Tổng số lớp</t>
+          <t>Tổng số học sinh</t>
         </is>
       </c>
       <c r="C40" s="32" t="inlineStr"/>
-      <c r="D40" s="11" t="inlineStr">
-        <is>
-          <t>Để đối chiếu với tệp CSDL ngành</t>
-        </is>
-      </c>
+      <c r="D40" s="11" t="inlineStr"/>
     </row>
     <row r="41" ht="24" customHeight="1">
       <c r="A41" s="31" t="inlineStr">
         <is>
-          <t>SO_HOC_SINH</t>
+          <t>SO_CBGV</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Tổng số học sinh</t>
+          <t>Tổng số cán bộ quản lý, giáo viên, nhân viên</t>
         </is>
       </c>
       <c r="C41" s="32" t="inlineStr"/>
@@ -2000,176 +2002,162 @@
     <row r="42" ht="24" customHeight="1">
       <c r="A42" s="31" t="inlineStr">
         <is>
-          <t>SO_CBGV</t>
+          <t>SO_DIEM_TRUONG</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Tổng số cán bộ quản lý, giáo viên, nhân viên</t>
+          <t>Số cơ sở, phân hiệu, điểm trường</t>
         </is>
       </c>
       <c r="C42" s="32" t="inlineStr"/>
-      <c r="D42" s="11" t="inlineStr"/>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>Trường một địa điểm ghi 1</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="24" customHeight="1">
       <c r="A43" s="31" t="inlineStr">
         <is>
-          <t>SO_DIEM_TRUONG</t>
+          <t>CO_SAP_NHAP</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Số cơ sở, phân hiệu, điểm trường</t>
+          <t>Trường có sáp nhập từ các trường khác không</t>
         </is>
       </c>
       <c r="C43" s="32" t="inlineStr"/>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Trường một địa điểm ghi 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="24" customHeight="1">
-      <c r="A44" s="31" t="inlineStr">
-        <is>
-          <t>CO_SAP_NHAP</t>
-        </is>
-      </c>
-      <c r="B44" s="10" t="inlineStr">
-        <is>
-          <t>Trường có sáp nhập từ các trường khác không</t>
-        </is>
-      </c>
-      <c r="C44" s="32" t="inlineStr"/>
-      <c r="D44" s="11" t="inlineStr">
-        <is>
           <t>Chọn Có / Không — nếu Có, điền thêm phần C trang 5</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>Đ. NHẬN DIỆN VÀ QUẢN TRỊ</t>
         </is>
       </c>
-      <c r="B45" s="16" t="n"/>
-      <c r="C45" s="16" t="n"/>
-      <c r="D45" s="17" t="n"/>
+      <c r="B44" s="16" t="n"/>
+      <c r="C44" s="16" t="n"/>
+      <c r="D44" s="17" t="n"/>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="31" t="inlineStr">
+        <is>
+          <t>SLOGAN</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Khẩu hiệu, phương châm của trường</t>
+        </is>
+      </c>
+      <c r="C45" s="32" t="inlineStr"/>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>Ví dụ: Vững bước tương lai - Tự tin hội nhập</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="31" t="inlineStr">
         <is>
-          <t>SLOGAN</t>
+          <t>MAU_CHU_DAO</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Khẩu hiệu, phương châm của trường</t>
+          <t>Màu chủ đạo mong muốn cho trang</t>
         </is>
       </c>
       <c r="C46" s="32" t="inlineStr"/>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Ví dụ: Vững bước tương lai - Tự tin hội nhập</t>
+          <t>Ghi tên màu: xanh dương, xanh lá, đỏ đô…</t>
         </is>
       </c>
     </row>
     <row r="47" ht="24" customHeight="1">
       <c r="A47" s="31" t="inlineStr">
         <is>
-          <t>MAU_CHU_DAO</t>
+          <t>QUAN_TRI_TEN</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Màu chủ đạo mong muốn cho trang</t>
+          <t>Người phụ trách hệ thống phía trường — họ tên</t>
         </is>
       </c>
       <c r="C47" s="32" t="inlineStr"/>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>Ghi tên màu: xanh dương, xanh lá, đỏ đô…</t>
+          <t>Người được cấp quyền quản trị, tập huấn kỹ nhất</t>
         </is>
       </c>
     </row>
     <row r="48" ht="24" customHeight="1">
       <c r="A48" s="31" t="inlineStr">
         <is>
-          <t>QUAN_TRI_TEN</t>
+          <t>QUAN_TRI_EMAIL</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Người phụ trách hệ thống phía trường — họ tên</t>
+          <t>Người phụ trách hệ thống — thư điện tử</t>
         </is>
       </c>
       <c r="C48" s="32" t="inlineStr"/>
-      <c r="D48" s="11" t="inlineStr">
-        <is>
-          <t>Người được cấp quyền quản trị, tập huấn kỹ nhất</t>
-        </is>
-      </c>
+      <c r="D48" s="11" t="inlineStr"/>
     </row>
     <row r="49" ht="24" customHeight="1">
       <c r="A49" s="31" t="inlineStr">
         <is>
-          <t>QUAN_TRI_EMAIL</t>
+          <t>CO_DRIVE</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Người phụ trách hệ thống — thư điện tử</t>
+          <t>Trường đã có Google Drive dùng chung chưa</t>
         </is>
       </c>
       <c r="C49" s="32" t="inlineStr"/>
-      <c r="D49" s="11" t="inlineStr"/>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Chọn Có / Không</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="24" customHeight="1">
       <c r="A50" s="31" t="inlineStr">
         <is>
-          <t>CO_DRIVE</t>
+          <t>LINK_DRIVE</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Trường đã có Google Drive dùng chung chưa</t>
+          <t>Đường dẫn thư mục Drive hiện có (nếu có)</t>
         </is>
       </c>
       <c r="C50" s="32" t="inlineStr"/>
-      <c r="D50" s="11" t="inlineStr">
-        <is>
-          <t>Chọn Có / Không</t>
-        </is>
-      </c>
+      <c r="D50" s="11" t="inlineStr"/>
     </row>
     <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="31" t="inlineStr">
-        <is>
-          <t>LINK_DRIVE</t>
-        </is>
-      </c>
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t>Đường dẫn thư mục Drive hiện có (nếu có)</t>
-        </is>
-      </c>
-      <c r="C51" s="32" t="inlineStr"/>
-      <c r="D51" s="11" t="inlineStr"/>
-    </row>
-    <row r="52" ht="24" customHeight="1">
-      <c r="A52" s="33" t="inlineStr">
+      <c r="A51" s="33" t="inlineStr">
         <is>
           <t>GHI_CHU_TRUONG</t>
         </is>
       </c>
-      <c r="B52" s="25" t="inlineStr">
+      <c r="B51" s="25" t="inlineStr">
         <is>
           <t>Nguyện vọng khác của nhà trường</t>
         </is>
       </c>
-      <c r="C52" s="34" t="inlineStr"/>
-      <c r="D52" s="35" t="inlineStr">
+      <c r="C51" s="34" t="inlineStr"/>
+      <c r="D51" s="35" t="inlineStr">
         <is>
           <t>Ghi tự do</t>
         </is>
@@ -2179,20 +2167,20 @@
   <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A45:D45"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A29:D29"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A44:D44"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="C31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>DM!$D$1:$D$3</formula1>
     </dataValidation>
     <dataValidation sqref="C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>DM!$G$1:$G$3</formula1>
     </dataValidation>
-    <dataValidation sqref="C35 C44 C50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C34 C43 C49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>DM!$C$1:$C$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -2247,6 +2235,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2477,6 +2466,7 @@
       <c r="K12" s="44" t="n"/>
       <c r="L12" s="45" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="46" t="inlineStr">
         <is>
@@ -3240,6 +3230,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="28" t="inlineStr">
         <is>
@@ -3811,6 +3802,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="28" t="inlineStr">
         <is>
@@ -3965,7 +3957,7 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Đoàn TNCS, Đội TNTP &amp; Sao Nhi đồng</t>
+          <t>Đoàn TNCS, Đội TNTP - Sao Nhi đồng</t>
         </is>
       </c>
       <c r="E9" s="32" t="inlineStr"/>
@@ -4222,6 +4214,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="28" t="inlineStr">
         <is>
@@ -5629,7 +5622,7 @@
       <c r="F59" s="32" t="inlineStr"/>
       <c r="G59" s="10" t="inlineStr">
         <is>
-          <t>Công đoàn</t>
+          <t>Văn phòng</t>
         </is>
       </c>
       <c r="H59" s="48" t="inlineStr"/>

</xml_diff>